<commit_message>
Actualiza notas de pares del CR-302
</commit_message>
<xml_diff>
--- a/docs/Notas de pares.xlsx
+++ b/docs/Notas de pares.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Laboratorio_24\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\casa2\Desktop\LicitacionesUV\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1A580DA-5DD9-4E69-ABC9-4C58C8C394E1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1CD7FF0-91EF-42E6-BC07-F1282C657EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{5989487C-A4E6-4BC1-B570-30DE59AF3F3D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5989487C-A4E6-4BC1-B570-30DE59AF3F3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,9 +36,6 @@
     <t>Vicente Saa</t>
   </si>
   <si>
-    <t>Benjamin Tulazo</t>
-  </si>
-  <si>
     <t>Wilson Jara</t>
   </si>
   <si>
@@ -48,7 +45,10 @@
     <t xml:space="preserve">Vicente Garcia </t>
   </si>
   <si>
-    <t>x|</t>
+    <t>Benjamin lazo</t>
+  </si>
+  <si>
+    <t>70|</t>
   </si>
 </sst>
 </file>
@@ -119,12 +119,12 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -143,9 +143,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -183,7 +183,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -289,7 +289,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -431,7 +431,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -443,227 +443,227 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="2" t="s">
+      <c r="F2" s="3"/>
+      <c r="G2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="2">
+        <v>70</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4"/>
+      <c r="G3" s="2">
+        <v>70</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3" s="4"/>
+      <c r="K3" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="2">
+        <v>70</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="4"/>
+      <c r="G4" s="2">
+        <v>70</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4"/>
+      <c r="K4" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="1"/>
-      <c r="K2" s="2" t="s">
+      <c r="B5" s="4"/>
+      <c r="C5" s="2">
+        <v>70</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="4"/>
+      <c r="G5" s="2">
+        <v>70</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="4"/>
+      <c r="K5" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="2">
+        <v>70</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="4"/>
+      <c r="G6" s="2">
+        <v>70</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J6" s="4"/>
+      <c r="K6" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="E10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="4">
-        <v>70</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="B11" s="4"/>
+      <c r="C11" s="2">
+        <v>70</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="4"/>
+      <c r="G11" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="2">
+        <v>70</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" s="4"/>
+      <c r="G12" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="4">
-        <v>70</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="J3" s="3"/>
-      <c r="K3" s="4">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="B13" s="4"/>
+      <c r="C13" s="2">
+        <v>70</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="4">
-        <v>70</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="4">
-        <v>70</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="4">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="F13" s="4"/>
+      <c r="G13" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="4">
-        <v>70</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="4">
-        <v>70</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="J5" s="3"/>
-      <c r="K5" s="4">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="B14" s="4"/>
+      <c r="C14" s="2">
+        <v>70</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="4">
-        <v>70</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="4">
-        <v>70</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="J6" s="3"/>
-      <c r="K6" s="4">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="4">
-        <v>70</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="4">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="4">
-        <v>70</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="4">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="4">
-        <v>70</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="4">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="4">
-        <v>70</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="4" t="s">
+      <c r="F14" s="4"/>
+      <c r="G14" s="2" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E14:F14"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>